<commit_message>
added spm bands extractor
</commit_message>
<xml_diff>
--- a/sampledata/2020/WMS_Rrs_micasense_SPM.xlsx
+++ b/sampledata/2020/WMS_Rrs_micasense_SPM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MSU\SPM\Field Data\2020\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\codes\radiometer_processor\sampledata\2020\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F63CE79C-F31B-494E-A570-78D6D41D9981}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF33F79-6959-4F45-8C44-8CD322D0B023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -741,6 +741,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -748,7 +749,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1401,6 +1401,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1408,7 +1409,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2401,6 +2401,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2408,7 +2409,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2984,6 +2984,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2991,7 +2992,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6450,16 +6450,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>396240</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>91440</xdr:colOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>388620</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:rowOff>15240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6593,9 +6593,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -6633,9 +6633,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -6668,26 +6668,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -6720,26 +6703,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>